<commit_message>
Fix #6: Standardize Prior Year term values to 3-term system (FY/S1/S2)
- Changed 'ALL' → 'FY' (8 rows) — these are full-year courses
- Changed 'S1, S2' → 'FY' (291 rows) — courses meeting both semesters = full-year
- Kept standalone 'S1' (70 rows) and 'S2' (74 rows) unchanged
- Total: 299 cells changed in Grading Periods column (col 8)
- Prior Year now uses same 3-term vocabulary as engine and all other templates
- Per JC directive: school has 3 terms only (FY=5.0cr, S1=2.5cr, S2=2.5cr)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/202526_Master_Schedule_With_Teacher_ID.xlsx
+++ b/templates/202526_Master_Schedule_With_Teacher_ID.xlsx
@@ -1304,7 +1304,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5556,7 +5556,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -6804,7 +6804,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -6900,7 +6900,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -6948,7 +6948,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -7476,7 +7476,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7812,7 +7812,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -7860,7 +7860,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -8052,7 +8052,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -8196,7 +8196,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -8292,7 +8292,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -8916,7 +8916,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -9108,7 +9108,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -9156,7 +9156,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -9348,7 +9348,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -9396,7 +9396,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -9573,7 +9573,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -9669,7 +9669,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -9717,7 +9717,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -10033,7 +10033,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -10081,7 +10081,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -10753,7 +10753,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -12913,7 +12913,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -13057,7 +13057,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -13153,7 +13153,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -13249,7 +13249,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -13297,7 +13297,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -13393,7 +13393,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -13537,7 +13537,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -13585,7 +13585,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -13633,7 +13633,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -13777,7 +13777,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -13873,7 +13873,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -13921,7 +13921,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -13969,7 +13969,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -14017,7 +14017,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -14065,7 +14065,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -14113,7 +14113,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -14257,7 +14257,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -14305,7 +14305,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -14353,7 +14353,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -14401,7 +14401,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -14497,7 +14497,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -14545,7 +14545,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -14593,7 +14593,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -14641,7 +14641,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -14689,7 +14689,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -14737,7 +14737,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -14929,7 +14929,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -14977,7 +14977,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -15025,7 +15025,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -15073,7 +15073,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -15169,7 +15169,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -15217,7 +15217,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -15265,7 +15265,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -15313,7 +15313,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
@@ -15361,7 +15361,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -15409,7 +15409,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -15457,7 +15457,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -15553,7 +15553,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -15601,7 +15601,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -15649,7 +15649,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -15697,7 +15697,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -15745,7 +15745,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -15793,7 +15793,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -15841,7 +15841,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -15937,7 +15937,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I324" t="inlineStr">
@@ -15985,7 +15985,7 @@
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I325" t="inlineStr">
@@ -16033,7 +16033,7 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I326" t="inlineStr">
@@ -16081,7 +16081,7 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I327" t="inlineStr">
@@ -16225,7 +16225,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -16546,7 +16546,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -16670,7 +16670,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -16718,7 +16718,7 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
@@ -16862,7 +16862,7 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -16958,7 +16958,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -17006,7 +17006,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -17054,7 +17054,7 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -17102,7 +17102,7 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
@@ -17150,7 +17150,7 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
@@ -17389,7 +17389,7 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J400" t="inlineStr">
@@ -17427,7 +17427,7 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J401" t="inlineStr">
@@ -17465,7 +17465,7 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J402" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J403" t="inlineStr">
@@ -17541,7 +17541,7 @@
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J404" t="inlineStr">
@@ -17579,7 +17579,7 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
@@ -17617,7 +17617,7 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J406" t="inlineStr">
@@ -17655,7 +17655,7 @@
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
@@ -17693,7 +17693,7 @@
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J408" t="inlineStr">
@@ -17731,7 +17731,7 @@
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J409" t="inlineStr">
@@ -17769,7 +17769,7 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J410" t="inlineStr">
@@ -17807,7 +17807,7 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J411" t="inlineStr">
@@ -17845,7 +17845,7 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J412" t="inlineStr">
@@ -17883,7 +17883,7 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J413" t="inlineStr">
@@ -17921,7 +17921,7 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J414" t="inlineStr">
@@ -17959,7 +17959,7 @@
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J415" t="inlineStr">
@@ -17997,7 +17997,7 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J416" t="inlineStr">
@@ -18035,7 +18035,7 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J417" t="inlineStr">
@@ -18073,7 +18073,7 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J418" t="inlineStr">
@@ -18111,7 +18111,7 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J419" t="inlineStr">
@@ -18149,7 +18149,7 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J420" t="inlineStr">
@@ -18187,7 +18187,7 @@
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J421" t="inlineStr">
@@ -18225,7 +18225,7 @@
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J422" t="inlineStr">
@@ -18263,7 +18263,7 @@
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J423" t="inlineStr">
@@ -18301,7 +18301,7 @@
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J424" t="inlineStr">
@@ -18339,7 +18339,7 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J425" t="inlineStr">
@@ -18377,7 +18377,7 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J426" t="inlineStr">
@@ -18415,7 +18415,7 @@
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J427" t="inlineStr">
@@ -18453,7 +18453,7 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J428" t="inlineStr">
@@ -18491,7 +18491,7 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J429" t="inlineStr">
@@ -18529,7 +18529,7 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J430" t="inlineStr">
@@ -18567,7 +18567,7 @@
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J431" t="inlineStr">
@@ -18605,7 +18605,7 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J432" t="inlineStr">
@@ -18643,7 +18643,7 @@
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J433" t="inlineStr">
@@ -18681,7 +18681,7 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J434" t="inlineStr">
@@ -18719,7 +18719,7 @@
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I435" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I436" t="inlineStr">
@@ -18805,7 +18805,7 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
@@ -18848,7 +18848,7 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
@@ -18891,7 +18891,7 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I439" t="inlineStr">
@@ -18934,7 +18934,7 @@
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I440" t="inlineStr">
@@ -18977,7 +18977,7 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
@@ -19020,7 +19020,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J442" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J443" t="inlineStr">
@@ -19096,7 +19096,7 @@
       </c>
       <c r="H444" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J444" t="inlineStr">
@@ -19134,7 +19134,7 @@
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J445" t="inlineStr">
@@ -19172,7 +19172,7 @@
       </c>
       <c r="H446" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J446" t="inlineStr">
@@ -19210,7 +19210,7 @@
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J447" t="inlineStr">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="J448" t="inlineStr">
@@ -19387,7 +19387,7 @@
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I451" t="inlineStr">
@@ -19435,7 +19435,7 @@
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I452" t="inlineStr">
@@ -19483,7 +19483,7 @@
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I453" t="inlineStr">
@@ -19531,7 +19531,7 @@
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I454" t="inlineStr">
@@ -19579,7 +19579,7 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
@@ -19627,7 +19627,7 @@
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I456" t="inlineStr">
@@ -19675,7 +19675,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I458" t="inlineStr">
@@ -19771,7 +19771,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -19819,7 +19819,7 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
@@ -19867,7 +19867,7 @@
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I461" t="inlineStr">
@@ -19915,7 +19915,7 @@
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I462" t="inlineStr">
@@ -19963,7 +19963,7 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I464" t="inlineStr">
@@ -20059,7 +20059,7 @@
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I465" t="inlineStr">
@@ -20107,7 +20107,7 @@
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I466" t="inlineStr">
@@ -20155,7 +20155,7 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
@@ -20203,7 +20203,7 @@
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I468" t="inlineStr">
@@ -20251,7 +20251,7 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
@@ -20299,7 +20299,7 @@
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I470" t="inlineStr">
@@ -20347,7 +20347,7 @@
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I471" t="inlineStr">
@@ -20395,7 +20395,7 @@
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
@@ -20443,7 +20443,7 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
@@ -20491,7 +20491,7 @@
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I474" t="inlineStr">
@@ -20539,7 +20539,7 @@
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I475" t="inlineStr">
@@ -20587,7 +20587,7 @@
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I476" t="inlineStr">
@@ -20635,7 +20635,7 @@
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I477" t="inlineStr">
@@ -20683,7 +20683,7 @@
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>S1, S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="I478" t="inlineStr">

</xml_diff>